<commit_message>
Refine unit tests on model simulation, regenerate simulation data
</commit_message>
<xml_diff>
--- a/_ground_truth/true_params.xlsx
+++ b/_ground_truth/true_params.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10309"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/selinapi/Repositories/tutorial_cancer_modeling_des/_ground_truth/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8971759E-B15B-1F4D-B5E5-B694D68782B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F06D3993-1DC6-9A4E-876D-03ACDE4A4919}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34860" yWindow="-80" windowWidth="30240" windowHeight="17540" xr2:uid="{3F2257C7-EED0-BA4B-BED8-66F74100CF01}"/>
+    <workbookView xWindow="15120" yWindow="760" windowWidth="15120" windowHeight="17760" xr2:uid="{3F2257C7-EED0-BA4B-BED8-66F74100CF01}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -56,9 +56,6 @@
     <t>rate</t>
   </si>
   <si>
-    <t>exponential</t>
-  </si>
-  <si>
     <t>var_name</t>
   </si>
   <si>
@@ -108,6 +105,9 @@
   </si>
   <si>
     <t>p_cancer</t>
+  </si>
+  <si>
+    <t>exp</t>
   </si>
 </sst>
 </file>
@@ -495,27 +495,27 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" t="s">
         <v>7</v>
       </c>
-      <c r="B1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>8</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>9</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>10</v>
-      </c>
-      <c r="F1" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>1</v>
@@ -533,7 +533,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>1</v>
@@ -551,7 +551,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>1</v>
@@ -569,7 +569,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>1</v>
@@ -587,13 +587,13 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>16</v>
       </c>
       <c r="E6" s="1">
         <f>1/16</f>
@@ -648,7 +648,7 @@
       </c>
       <c r="B9" s="1"/>
       <c r="C9" s="1" t="s">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>5</v>
@@ -663,7 +663,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B10" s="1">
         <v>1</v>
@@ -680,7 +680,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B11" s="1">
         <v>2</v>
@@ -697,7 +697,7 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B12" s="1">
         <v>3</v>
@@ -714,7 +714,7 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B13" s="1">
         <v>4</v>
@@ -731,7 +731,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B14" s="1">
         <v>1</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B15" s="1">
         <v>2</v>
@@ -765,7 +765,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B16" s="1">
         <v>3</v>
@@ -782,7 +782,7 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B17" s="1">
         <v>4</v>
@@ -800,11 +800,11 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B18" s="1"/>
       <c r="C18" s="1" t="s">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>5</v>
@@ -819,11 +819,11 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B19" s="1"/>
       <c r="C19" s="1" t="s">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>5</v>
@@ -838,11 +838,11 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B20" s="1"/>
       <c r="C20" s="1" t="s">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>5</v>
@@ -857,11 +857,11 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B21" s="1"/>
       <c r="C21" s="1" t="s">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>5</v>

</xml_diff>